<commit_message>
Update CHANGELOG with performance improvements and bug fixes. Consolidated Meetings V2 counts calculation to reduce database load, fixed PDF viewer race conditions, and enhanced polling logic in MeetingV2Detail. Added new utility functions for bulk extract run status and improved PDF rendering management. Updated middleware for session cookie handling and added new tests for meeting status polling.
</commit_message>
<xml_diff>
--- a/docs/building-link-data.xlsx
+++ b/docs/building-link-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pgart\Development\Condo board\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A71EF452-7633-40D2-A666-AE30CBA265F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5495D90C-85C1-4961-879F-D5B72F8E11F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1356,10 +1356,10 @@
   <cols>
     <col min="2" max="2" width="23.8125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.8125" customWidth="1"/>
-    <col min="4" max="4" width="16.3125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.75" customWidth="1"/>
+    <col min="4" max="4" width="16.3125" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="15.75" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="7" max="7" width="9.9375" customWidth="1"/>
     <col min="8" max="8" width="27.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.6875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="26.1875" bestFit="1" customWidth="1"/>
@@ -1420,43 +1420,43 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A2">
-        <v>1</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
-        <v>234</v>
+        <v>268</v>
       </c>
       <c r="C2" t="s">
-        <v>286</v>
+        <v>297</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>294</v>
       </c>
       <c r="E2" t="s">
         <v>221</v>
       </c>
       <c r="F2" t="s">
-        <v>222</v>
+        <v>231</v>
       </c>
       <c r="G2">
-        <v>32</v>
+        <v>-1</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="I2" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="J2" t="s">
-        <v>15</v>
+        <v>151</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>152</v>
       </c>
       <c r="L2" t="s">
-        <v>17</v>
+        <v>153</v>
       </c>
       <c r="M2" t="s">
-        <v>18</v>
+        <v>154</v>
       </c>
       <c r="N2" t="s">
         <v>19</v>
@@ -1520,43 +1520,43 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A4">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C4" t="s">
-        <v>235</v>
+        <v>287</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
         <v>221</v>
       </c>
       <c r="F4" t="s">
-        <v>224</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>305</v>
+        <v>222</v>
+      </c>
+      <c r="G4">
+        <v>-1</v>
       </c>
       <c r="H4" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="I4" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="K4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="L4" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="M4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N4" t="s">
         <v>19</v>
@@ -1620,40 +1620,40 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A6">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
         <v>221</v>
       </c>
       <c r="F6" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G6">
-        <v>32</v>
+        <v>-1</v>
       </c>
       <c r="H6" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="I6" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="J6" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="K6" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="L6" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="M6" t="s">
         <v>18</v>
@@ -1665,7 +1665,7 @@
         <v>19</v>
       </c>
       <c r="P6" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -1720,22 +1720,22 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A8">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="C8" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="E8" t="s">
         <v>221</v>
       </c>
       <c r="F8" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="G8">
         <v>-1</v>
@@ -1744,16 +1744,16 @@
         <v>34</v>
       </c>
       <c r="I8" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="J8" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="K8" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="L8" t="s">
-        <v>30</v>
+        <v>76</v>
       </c>
       <c r="M8" t="s">
         <v>18</v>
@@ -1870,37 +1870,43 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A11">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>251</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>290</v>
       </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="E11" t="s">
-        <v>42</v>
+        <v>221</v>
+      </c>
+      <c r="F11" t="s">
+        <v>227</v>
+      </c>
+      <c r="G11">
+        <v>-1</v>
       </c>
       <c r="H11" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>84</v>
       </c>
       <c r="J11" t="s">
-        <v>19</v>
+        <v>85</v>
       </c>
       <c r="K11" t="s">
-        <v>19</v>
+        <v>86</v>
       </c>
       <c r="L11" t="s">
-        <v>19</v>
+        <v>87</v>
       </c>
       <c r="M11" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="N11" t="s">
         <v>19</v>
@@ -1914,40 +1920,40 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A12">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="C12" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D12" t="s">
-        <v>45</v>
+        <v>93</v>
       </c>
       <c r="E12" t="s">
         <v>221</v>
       </c>
       <c r="F12" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G12">
         <v>-1</v>
       </c>
       <c r="H12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I12" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="J12" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="K12" t="s">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="L12" t="s">
-        <v>47</v>
+        <v>81</v>
       </c>
       <c r="M12" t="s">
         <v>18</v>
@@ -1959,7 +1965,7 @@
         <v>19</v>
       </c>
       <c r="P12" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -2014,40 +2020,40 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A14">
-        <v>13</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
       <c r="C14" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D14" t="s">
-        <v>50</v>
+        <v>121</v>
       </c>
       <c r="E14" t="s">
         <v>221</v>
       </c>
       <c r="F14" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="G14">
-        <v>32</v>
+        <v>-1</v>
       </c>
       <c r="H14" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="I14" t="s">
-        <v>46</v>
+        <v>116</v>
       </c>
       <c r="J14" t="s">
-        <v>19</v>
+        <v>122</v>
       </c>
       <c r="K14" t="s">
-        <v>19</v>
+        <v>123</v>
       </c>
       <c r="L14" t="s">
-        <v>19</v>
+        <v>124</v>
       </c>
       <c r="M14" t="s">
         <v>18</v>
@@ -2059,7 +2065,7 @@
         <v>19</v>
       </c>
       <c r="P14" t="s">
-        <v>48</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -2114,40 +2120,40 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A16">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>241</v>
+        <v>262</v>
       </c>
       <c r="C16" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D16" t="s">
-        <v>54</v>
+        <v>133</v>
       </c>
       <c r="E16" t="s">
         <v>221</v>
       </c>
       <c r="F16" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G16">
-        <v>32</v>
+        <v>-1</v>
       </c>
       <c r="H16" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="I16" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="J16" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="K16" t="s">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="L16" t="s">
-        <v>49</v>
+        <v>100</v>
       </c>
       <c r="M16" t="s">
         <v>18</v>
@@ -2214,43 +2220,43 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A18">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="B18" t="s">
-        <v>242</v>
+        <v>264</v>
       </c>
       <c r="C18" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D18" t="s">
-        <v>59</v>
+        <v>138</v>
       </c>
       <c r="E18" t="s">
         <v>221</v>
       </c>
       <c r="F18" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H18" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="I18" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J18" t="s">
-        <v>62</v>
+        <v>19</v>
       </c>
       <c r="K18" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="L18" t="s">
         <v>19</v>
       </c>
       <c r="M18" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N18" t="s">
         <v>19</v>
@@ -2259,7 +2265,7 @@
         <v>19</v>
       </c>
       <c r="P18" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -2314,43 +2320,43 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A20">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>244</v>
+        <v>265</v>
       </c>
       <c r="C20" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D20" t="s">
-        <v>68</v>
+        <v>142</v>
       </c>
       <c r="E20" t="s">
         <v>221</v>
       </c>
       <c r="F20" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H20" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="I20" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J20" t="s">
-        <v>62</v>
+        <v>19</v>
       </c>
       <c r="K20" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="L20" t="s">
         <v>19</v>
       </c>
       <c r="M20" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N20" t="s">
         <v>19</v>
@@ -2359,7 +2365,7 @@
         <v>19</v>
       </c>
       <c r="P20" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -2414,43 +2420,43 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A22">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>245</v>
+        <v>266</v>
       </c>
       <c r="C22" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D22" t="s">
-        <v>70</v>
+        <v>145</v>
       </c>
       <c r="E22" t="s">
         <v>221</v>
       </c>
       <c r="F22" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G22">
-        <v>32</v>
+        <v>-1</v>
       </c>
       <c r="H22" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="I22" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="J22" t="s">
-        <v>62</v>
+        <v>19</v>
       </c>
       <c r="K22" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="L22" t="s">
         <v>19</v>
       </c>
       <c r="M22" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N22" t="s">
         <v>19</v>
@@ -2459,7 +2465,7 @@
         <v>19</v>
       </c>
       <c r="P22" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -2564,43 +2570,43 @@
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A25">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="B25" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="C25" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="D25" t="s">
-        <v>71</v>
+        <v>295</v>
       </c>
       <c r="E25" t="s">
         <v>221</v>
       </c>
       <c r="F25" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="G25">
-        <v>32</v>
+        <v>-1</v>
       </c>
       <c r="H25" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="I25" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="J25" t="s">
-        <v>19</v>
+        <v>156</v>
       </c>
       <c r="K25" t="s">
-        <v>19</v>
+        <v>157</v>
       </c>
       <c r="L25" t="s">
-        <v>73</v>
+        <v>141</v>
       </c>
       <c r="M25" t="s">
-        <v>74</v>
+        <v>154</v>
       </c>
       <c r="N25" t="s">
         <v>19</v>
@@ -2664,22 +2670,22 @@
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A27">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>249</v>
+        <v>270</v>
       </c>
       <c r="C27" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="D27" t="s">
-        <v>75</v>
+        <v>296</v>
       </c>
       <c r="E27" t="s">
         <v>221</v>
       </c>
       <c r="F27" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="G27">
         <v>-1</v>
@@ -2688,16 +2694,16 @@
         <v>34</v>
       </c>
       <c r="I27" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="J27" t="s">
         <v>19</v>
       </c>
       <c r="K27" t="s">
-        <v>19</v>
+        <v>161</v>
       </c>
       <c r="L27" t="s">
-        <v>76</v>
+        <v>162</v>
       </c>
       <c r="M27" t="s">
         <v>18</v>
@@ -2714,40 +2720,40 @@
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A28">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="B28" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="C28" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="D28" t="s">
-        <v>77</v>
+        <v>171</v>
       </c>
       <c r="E28" t="s">
         <v>221</v>
       </c>
       <c r="F28" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="G28">
-        <v>32</v>
+        <v>-1</v>
       </c>
       <c r="H28" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="I28" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="J28" t="s">
-        <v>79</v>
+        <v>166</v>
       </c>
       <c r="K28" t="s">
-        <v>80</v>
+        <v>172</v>
       </c>
       <c r="L28" t="s">
-        <v>81</v>
+        <v>173</v>
       </c>
       <c r="M28" t="s">
         <v>18</v>
@@ -2814,22 +2820,22 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A30">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="B30" t="s">
-        <v>251</v>
+        <v>279</v>
       </c>
       <c r="C30" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="D30" t="s">
-        <v>83</v>
+        <v>194</v>
       </c>
       <c r="E30" t="s">
         <v>221</v>
       </c>
       <c r="F30" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="G30">
         <v>-1</v>
@@ -2838,16 +2844,16 @@
         <v>34</v>
       </c>
       <c r="I30" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="J30" t="s">
-        <v>85</v>
+        <v>158</v>
       </c>
       <c r="K30" t="s">
-        <v>86</v>
+        <v>195</v>
       </c>
       <c r="L30" t="s">
-        <v>87</v>
+        <v>47</v>
       </c>
       <c r="M30" t="s">
         <v>18</v>
@@ -2914,40 +2920,40 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A32">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="B32" t="s">
-        <v>252</v>
+        <v>284</v>
       </c>
       <c r="C32" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="D32" t="s">
-        <v>89</v>
+        <v>300</v>
       </c>
       <c r="E32" t="s">
         <v>221</v>
       </c>
       <c r="F32" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="G32">
-        <v>32</v>
+        <v>-1</v>
       </c>
       <c r="H32" t="s">
-        <v>13</v>
+        <v>208</v>
       </c>
       <c r="I32" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="J32" t="s">
-        <v>90</v>
+        <v>209</v>
       </c>
       <c r="K32" t="s">
-        <v>91</v>
+        <v>210</v>
       </c>
       <c r="L32" t="s">
-        <v>81</v>
+        <v>211</v>
       </c>
       <c r="M32" t="s">
         <v>18</v>
@@ -3014,22 +3020,22 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A34">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="B34" t="s">
-        <v>253</v>
+        <v>285</v>
       </c>
       <c r="C34" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="D34" t="s">
-        <v>93</v>
+        <v>301</v>
       </c>
       <c r="E34" t="s">
         <v>221</v>
       </c>
       <c r="F34" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="G34">
         <v>-1</v>
@@ -3038,16 +3044,16 @@
         <v>34</v>
       </c>
       <c r="I34" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="J34" t="s">
-        <v>94</v>
+        <v>215</v>
       </c>
       <c r="K34" t="s">
-        <v>95</v>
+        <v>216</v>
       </c>
       <c r="L34" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
       <c r="M34" t="s">
         <v>18</v>
@@ -3114,43 +3120,43 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A36">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="B36" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="C36" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D36" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="E36" t="s">
         <v>221</v>
       </c>
       <c r="F36" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G36">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="I36" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="J36" t="s">
-        <v>19</v>
+        <v>62</v>
       </c>
       <c r="K36" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="L36" t="s">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="M36" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N36" t="s">
         <v>19</v>
@@ -3159,7 +3165,7 @@
         <v>19</v>
       </c>
       <c r="P36" t="s">
-        <v>19</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -3364,43 +3370,43 @@
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A41">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="B41" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="C41" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D41" t="s">
-        <v>115</v>
+        <v>68</v>
       </c>
       <c r="E41" t="s">
         <v>221</v>
       </c>
       <c r="F41" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="G41">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="I41" t="s">
-        <v>116</v>
+        <v>61</v>
       </c>
       <c r="J41" t="s">
-        <v>117</v>
+        <v>62</v>
       </c>
       <c r="K41" t="s">
-        <v>118</v>
+        <v>63</v>
       </c>
       <c r="L41" t="s">
         <v>19</v>
       </c>
       <c r="M41" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N41" t="s">
         <v>19</v>
@@ -3409,7 +3415,7 @@
         <v>19</v>
       </c>
       <c r="P41" t="s">
-        <v>119</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -3464,43 +3470,43 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A43">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="B43" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="C43" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="D43" t="s">
-        <v>121</v>
+        <v>177</v>
       </c>
       <c r="E43" t="s">
         <v>221</v>
       </c>
       <c r="F43" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="G43">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="H43" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="I43" t="s">
-        <v>116</v>
+        <v>178</v>
       </c>
       <c r="J43" t="s">
-        <v>122</v>
+        <v>179</v>
       </c>
       <c r="K43" t="s">
-        <v>123</v>
+        <v>180</v>
       </c>
       <c r="L43" t="s">
-        <v>124</v>
+        <v>181</v>
       </c>
       <c r="M43" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N43" t="s">
         <v>19</v>
@@ -3509,7 +3515,7 @@
         <v>19</v>
       </c>
       <c r="P43" t="s">
-        <v>119</v>
+        <v>19</v>
       </c>
     </row>
     <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -3564,43 +3570,43 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A45">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="B45" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="C45" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="D45" t="s">
-        <v>126</v>
+        <v>185</v>
       </c>
       <c r="E45" t="s">
         <v>221</v>
       </c>
       <c r="F45" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G45">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="H45" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="I45" t="s">
-        <v>127</v>
+        <v>178</v>
       </c>
       <c r="J45" t="s">
-        <v>128</v>
+        <v>179</v>
       </c>
       <c r="K45" t="s">
-        <v>129</v>
+        <v>180</v>
       </c>
       <c r="L45" t="s">
-        <v>130</v>
+        <v>181</v>
       </c>
       <c r="M45" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N45" t="s">
         <v>19</v>
@@ -3664,40 +3670,40 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A47">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="B47" t="s">
-        <v>262</v>
+        <v>234</v>
       </c>
       <c r="C47" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="D47" t="s">
-        <v>133</v>
+        <v>12</v>
       </c>
       <c r="E47" t="s">
         <v>221</v>
       </c>
       <c r="F47" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="G47">
-        <v>-1</v>
+        <v>32</v>
       </c>
       <c r="H47" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I47" t="s">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="J47" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="K47" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="L47" t="s">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="M47" t="s">
         <v>18</v>
@@ -3764,22 +3770,22 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A49">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="B49" t="s">
-        <v>263</v>
+        <v>236</v>
       </c>
       <c r="C49" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D49" t="s">
-        <v>135</v>
+        <v>26</v>
       </c>
       <c r="E49" t="s">
         <v>221</v>
       </c>
       <c r="F49" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="G49">
         <v>32</v>
@@ -3788,16 +3794,16 @@
         <v>13</v>
       </c>
       <c r="I49" t="s">
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="J49" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="K49" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="L49" t="s">
-        <v>136</v>
+        <v>30</v>
       </c>
       <c r="M49" t="s">
         <v>18</v>
@@ -3864,16 +3870,16 @@
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A51">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="B51" t="s">
-        <v>264</v>
+        <v>240</v>
       </c>
       <c r="C51" t="s">
         <v>288</v>
       </c>
       <c r="D51" t="s">
-        <v>138</v>
+        <v>50</v>
       </c>
       <c r="E51" t="s">
         <v>221</v>
@@ -3882,10 +3888,10 @@
         <v>225</v>
       </c>
       <c r="G51">
-        <v>-1</v>
+        <v>32</v>
       </c>
       <c r="H51" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I51" t="s">
         <v>46</v>
@@ -3964,16 +3970,16 @@
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A53">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="B53" t="s">
-        <v>265</v>
+        <v>241</v>
       </c>
       <c r="C53" t="s">
         <v>288</v>
       </c>
       <c r="D53" t="s">
-        <v>142</v>
+        <v>54</v>
       </c>
       <c r="E53" t="s">
         <v>221</v>
@@ -3982,22 +3988,22 @@
         <v>225</v>
       </c>
       <c r="G53">
-        <v>-1</v>
+        <v>32</v>
       </c>
       <c r="H53" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I53" t="s">
         <v>46</v>
       </c>
       <c r="J53" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="K53" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="L53" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="M53" t="s">
         <v>18</v>
@@ -4009,7 +4015,7 @@
         <v>19</v>
       </c>
       <c r="P53" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
     </row>
     <row r="54" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -4064,43 +4070,43 @@
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A55">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="B55" t="s">
-        <v>266</v>
+        <v>245</v>
       </c>
       <c r="C55" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D55" t="s">
-        <v>145</v>
+        <v>70</v>
       </c>
       <c r="E55" t="s">
         <v>221</v>
       </c>
       <c r="F55" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G55">
-        <v>-1</v>
+        <v>32</v>
       </c>
       <c r="H55" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I55" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="J55" t="s">
-        <v>19</v>
+        <v>62</v>
       </c>
       <c r="K55" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="L55" t="s">
         <v>19</v>
       </c>
       <c r="M55" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N55" t="s">
         <v>19</v>
@@ -4109,7 +4115,7 @@
         <v>19</v>
       </c>
       <c r="P55" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
     </row>
     <row r="56" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -4214,43 +4220,43 @@
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A58">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="B58" t="s">
-        <v>268</v>
+        <v>247</v>
       </c>
       <c r="C58" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="D58" t="s">
-        <v>294</v>
+        <v>71</v>
       </c>
       <c r="E58" t="s">
         <v>221</v>
       </c>
       <c r="F58" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="G58">
-        <v>-2</v>
+        <v>32</v>
       </c>
       <c r="H58" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I58" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="J58" t="s">
-        <v>151</v>
+        <v>19</v>
       </c>
       <c r="K58" t="s">
-        <v>152</v>
+        <v>19</v>
       </c>
       <c r="L58" t="s">
-        <v>153</v>
+        <v>73</v>
       </c>
       <c r="M58" t="s">
-        <v>154</v>
+        <v>74</v>
       </c>
       <c r="N58" t="s">
         <v>19</v>
@@ -4314,43 +4320,43 @@
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A60">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="B60" t="s">
-        <v>269</v>
+        <v>250</v>
       </c>
       <c r="C60" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="D60" t="s">
-        <v>295</v>
+        <v>77</v>
       </c>
       <c r="E60" t="s">
         <v>221</v>
       </c>
       <c r="F60" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="G60">
-        <v>-1</v>
+        <v>32</v>
       </c>
       <c r="H60" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I60" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="J60" t="s">
-        <v>156</v>
+        <v>79</v>
       </c>
       <c r="K60" t="s">
-        <v>157</v>
+        <v>80</v>
       </c>
       <c r="L60" t="s">
-        <v>141</v>
+        <v>81</v>
       </c>
       <c r="M60" t="s">
-        <v>154</v>
+        <v>18</v>
       </c>
       <c r="N60" t="s">
         <v>19</v>
@@ -4414,40 +4420,40 @@
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A62">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="B62" t="s">
-        <v>270</v>
+        <v>252</v>
       </c>
       <c r="C62" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="D62" t="s">
-        <v>296</v>
+        <v>89</v>
       </c>
       <c r="E62" t="s">
         <v>221</v>
       </c>
       <c r="F62" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="G62">
-        <v>-1</v>
+        <v>32</v>
       </c>
       <c r="H62" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I62" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="J62" t="s">
-        <v>19</v>
+        <v>90</v>
       </c>
       <c r="K62" t="s">
-        <v>161</v>
+        <v>91</v>
       </c>
       <c r="L62" t="s">
-        <v>162</v>
+        <v>81</v>
       </c>
       <c r="M62" t="s">
         <v>18</v>
@@ -4514,22 +4520,22 @@
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A64">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="B64" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="C64" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="D64" t="s">
-        <v>165</v>
+        <v>99</v>
       </c>
       <c r="E64" t="s">
         <v>221</v>
       </c>
       <c r="F64" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="G64">
         <v>32</v>
@@ -4538,16 +4544,16 @@
         <v>13</v>
       </c>
       <c r="I64" t="s">
-        <v>46</v>
+        <v>72</v>
       </c>
       <c r="J64" t="s">
-        <v>166</v>
+        <v>19</v>
       </c>
       <c r="K64" t="s">
         <v>19</v>
       </c>
       <c r="L64" t="s">
-        <v>167</v>
+        <v>100</v>
       </c>
       <c r="M64" t="s">
         <v>18</v>
@@ -4614,40 +4620,40 @@
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A66">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="B66" t="s">
-        <v>272</v>
+        <v>259</v>
       </c>
       <c r="C66" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="D66" t="s">
-        <v>171</v>
+        <v>115</v>
       </c>
       <c r="E66" t="s">
         <v>221</v>
       </c>
       <c r="F66" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="G66">
-        <v>-1</v>
+        <v>32</v>
       </c>
       <c r="H66" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I66" t="s">
-        <v>46</v>
+        <v>116</v>
       </c>
       <c r="J66" t="s">
-        <v>166</v>
+        <v>117</v>
       </c>
       <c r="K66" t="s">
-        <v>172</v>
+        <v>118</v>
       </c>
       <c r="L66" t="s">
-        <v>173</v>
+        <v>19</v>
       </c>
       <c r="M66" t="s">
         <v>18</v>
@@ -4659,7 +4665,7 @@
         <v>19</v>
       </c>
       <c r="P66" t="s">
-        <v>19</v>
+        <v>119</v>
       </c>
     </row>
     <row r="67" spans="1:16" hidden="1" x14ac:dyDescent="0.5">
@@ -4714,43 +4720,43 @@
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A68">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="B68" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="C68" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="D68" t="s">
-        <v>177</v>
+        <v>126</v>
       </c>
       <c r="E68" t="s">
         <v>221</v>
       </c>
       <c r="F68" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="G68">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="H68" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="I68" t="s">
-        <v>178</v>
+        <v>127</v>
       </c>
       <c r="J68" t="s">
-        <v>179</v>
+        <v>128</v>
       </c>
       <c r="K68" t="s">
-        <v>180</v>
+        <v>129</v>
       </c>
       <c r="L68" t="s">
-        <v>181</v>
+        <v>130</v>
       </c>
       <c r="M68" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N68" t="s">
         <v>19</v>
@@ -4814,43 +4820,43 @@
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A70">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="B70" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="C70" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="D70" t="s">
-        <v>185</v>
+        <v>135</v>
       </c>
       <c r="E70" t="s">
         <v>221</v>
       </c>
       <c r="F70" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="G70">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="H70" t="s">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="I70" t="s">
-        <v>178</v>
+        <v>72</v>
       </c>
       <c r="J70" t="s">
-        <v>179</v>
+        <v>19</v>
       </c>
       <c r="K70" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="L70" t="s">
-        <v>181</v>
+        <v>136</v>
       </c>
       <c r="M70" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N70" t="s">
         <v>19</v>
@@ -4914,16 +4920,16 @@
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A72">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B72" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="C72" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D72" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
       <c r="E72" t="s">
         <v>221</v>
@@ -4938,19 +4944,19 @@
         <v>13</v>
       </c>
       <c r="I72" t="s">
-        <v>178</v>
+        <v>46</v>
       </c>
       <c r="J72" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
       <c r="K72" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="L72" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="M72" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="N72" t="s">
         <v>19</v>
@@ -5014,16 +5020,16 @@
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A74">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B74" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C74" t="s">
         <v>298</v>
       </c>
       <c r="D74" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E74" t="s">
         <v>221</v>
@@ -5041,10 +5047,10 @@
         <v>178</v>
       </c>
       <c r="J74" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="K74" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="L74" t="s">
         <v>181</v>
@@ -5164,16 +5170,16 @@
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A77">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B77" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C77" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D77" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E77" t="s">
         <v>221</v>
@@ -5188,19 +5194,19 @@
         <v>13</v>
       </c>
       <c r="I77" t="s">
-        <v>46</v>
+        <v>178</v>
       </c>
       <c r="J77" t="s">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="K77" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="L77" t="s">
-        <v>49</v>
+        <v>181</v>
       </c>
       <c r="M77" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N77" t="s">
         <v>19</v>
@@ -5214,16 +5220,16 @@
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A78">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B78" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C78" t="s">
         <v>297</v>
       </c>
       <c r="D78" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E78" t="s">
         <v>221</v>
@@ -5232,10 +5238,10 @@
         <v>231</v>
       </c>
       <c r="G78">
-        <v>-1</v>
+        <v>32</v>
       </c>
       <c r="H78" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="I78" t="s">
         <v>46</v>
@@ -5244,10 +5250,10 @@
         <v>158</v>
       </c>
       <c r="K78" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="L78" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="M78" t="s">
         <v>18</v>
@@ -5514,43 +5520,43 @@
     </row>
     <row r="84" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A84">
-        <v>83</v>
+        <v>3</v>
       </c>
       <c r="B84" t="s">
-        <v>284</v>
+        <v>235</v>
       </c>
       <c r="C84" t="s">
-        <v>302</v>
+        <v>235</v>
       </c>
       <c r="D84" t="s">
-        <v>300</v>
+        <v>23</v>
       </c>
       <c r="E84" t="s">
         <v>221</v>
       </c>
       <c r="F84" t="s">
-        <v>231</v>
-      </c>
-      <c r="G84">
-        <v>-1</v>
+        <v>224</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>305</v>
       </c>
       <c r="H84" t="s">
-        <v>208</v>
+        <v>24</v>
       </c>
       <c r="I84" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="J84" t="s">
-        <v>209</v>
+        <v>19</v>
       </c>
       <c r="K84" t="s">
-        <v>210</v>
+        <v>19</v>
       </c>
       <c r="L84" t="s">
-        <v>211</v>
+        <v>19</v>
       </c>
       <c r="M84" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N84" t="s">
         <v>19</v>
@@ -5614,43 +5620,37 @@
     </row>
     <row r="86" spans="1:16" x14ac:dyDescent="0.5">
       <c r="A86">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="B86" t="s">
-        <v>285</v>
+        <v>40</v>
       </c>
       <c r="C86" t="s">
-        <v>297</v>
+        <v>40</v>
       </c>
       <c r="D86" t="s">
-        <v>301</v>
+        <v>41</v>
       </c>
       <c r="E86" t="s">
-        <v>221</v>
-      </c>
-      <c r="F86" t="s">
-        <v>231</v>
-      </c>
-      <c r="G86">
-        <v>-1</v>
+        <v>42</v>
       </c>
       <c r="H86" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="I86" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="J86" t="s">
-        <v>215</v>
+        <v>19</v>
       </c>
       <c r="K86" t="s">
-        <v>216</v>
+        <v>19</v>
       </c>
       <c r="L86" t="s">
-        <v>141</v>
+        <v>19</v>
       </c>
       <c r="M86" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="N86" t="s">
         <v>19</v>
@@ -5814,10 +5814,13 @@
         <filter val="Studio 1"/>
       </filters>
     </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P88">
+      <sortCondition ref="G1:G89"/>
+    </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="H1:P89 D1:D57 B11 D64:D83 D88:D89" numberStoredAsText="1"/>
+    <ignoredError sqref="H1:P1 D1 D89 H89:P89" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>